<commit_message>
feat: implement loot selling and update related UI
</commit_message>
<xml_diff>
--- a/配置文档/GameConfig.xlsx
+++ b/配置文档/GameConfig.xlsx
@@ -3687,11 +3687,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>

</xml_diff>

<commit_message>
Add player analytics and refresh UI title icons
Track onboarding, sessions, currency spending, and receipt-backed purchases with analytics error isolation and persisted receipt metadata. Add analytics configuration and documentation, and update UI title icon assets.
</commit_message>
<xml_diff>
--- a/配置文档/GameConfig.xlsx
+++ b/配置文档/GameConfig.xlsx
@@ -1817,14 +1817,44 @@
       </s:c>
     </s:row>
     <s:row r="19" ht="24.6" customFormat="1" customHeight="1" s="11">
-      <s:c r="B19" s="12" t="n"/>
-      <s:c r="C19" s="12" t="n"/>
-      <s:c r="D19" s="13" t="n"/>
+      <s:c r="A19" s="12" t="inlineStr">
+        <s:is>
+          <s:t>string,bool</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B19" s="12" t="inlineStr">
+        <s:is>
+          <s:t>AnalyticsEnabled</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C19" s="12" t="b">
+        <s:v>1</s:v>
+      </s:c>
+      <s:c r="D19" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Analytics reporting enabled. Developer accounts are always excluded.</s:t>
+        </s:is>
+      </s:c>
     </s:row>
     <s:row r="20" ht="24.6" customFormat="1" customHeight="1" s="11">
-      <s:c r="B20" s="12" t="n"/>
-      <s:c r="C20" s="12" t="n"/>
-      <s:c r="D20" s="13" t="n"/>
+      <s:c r="A20" s="12" t="inlineStr">
+        <s:is>
+          <s:t>string,number_array</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B20" s="12" t="inlineStr">
+        <s:is>
+          <s:t>AnalyticsExcludedUserIds</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C20" s="12" t="n">
+        <s:v>2563885143</s:v>
+      </s:c>
+      <s:c r="D20" s="13" t="inlineStr">
+        <s:is>
+          <s:t>Excluded developer/test account UserIds, comma-separated numbers.</s:t>
+        </s:is>
+      </s:c>
     </s:row>
     <s:row r="21" ht="24.6" customFormat="1" customHeight="1" s="11">
       <s:c r="B21" s="12" t="n"/>

</xml_diff>

<commit_message>
Translate item names to English
</commit_message>
<xml_diff>
--- a/配置文档/GameConfig.xlsx
+++ b/配置文档/GameConfig.xlsx
@@ -3399,7 +3399,7 @@
       </s:c>
       <s:c r="C4" s="2" t="inlineStr">
         <s:is>
-          <s:t>打火机</s:t>
+          <s:t>Steel Nail</s:t>
         </s:is>
       </s:c>
       <s:c r="D4" s="2">
@@ -3431,7 +3431,7 @@
       </s:c>
       <s:c r="C5" s="2" t="inlineStr">
         <s:is>
-          <s:t>矿泉水</s:t>
+          <s:t>Tablet</s:t>
         </s:is>
       </s:c>
       <s:c r="D5" s="2">
@@ -3464,7 +3464,7 @@
       </s:c>
       <s:c r="C6" s="2" t="inlineStr">
         <s:is>
-          <s:t>纯净水</s:t>
+          <s:t>Capsule</s:t>
         </s:is>
       </s:c>
       <s:c r="D6" s="2">
@@ -3497,7 +3497,7 @@
       </s:c>
       <s:c r="C7" s="2" t="inlineStr">
         <s:is>
-          <s:t>苏打水</s:t>
+          <s:t>Dry Cell Battery</s:t>
         </s:is>
       </s:c>
       <s:c r="D7" s="2">
@@ -3530,7 +3530,7 @@
       </s:c>
       <s:c r="C8" s="2" t="inlineStr">
         <s:is>
-          <s:t>水桶</s:t>
+          <s:t>9V Battery</s:t>
         </s:is>
       </s:c>
       <s:c r="D8" s="2">
@@ -3560,7 +3560,7 @@
       </s:c>
       <s:c r="C9" s="2" t="inlineStr">
         <s:is>
-          <s:t>玻璃瓶</s:t>
+          <s:t>Crackers</s:t>
         </s:is>
       </s:c>
       <s:c r="D9" s="2">
@@ -3591,7 +3591,7 @@
       </s:c>
       <s:c r="C10" s="2" t="inlineStr">
         <s:is>
-          <s:t>啤酒瓶</s:t>
+          <s:t>Sandwich Crackers</s:t>
         </s:is>
       </s:c>
       <s:c r="D10" s="2">
@@ -3622,7 +3622,7 @@
       </s:c>
       <s:c r="C11" s="2" t="inlineStr">
         <s:is>
-          <s:t>红酒瓶</s:t>
+          <s:t>Packaged Crackers</s:t>
         </s:is>
       </s:c>
       <s:c r="D11" s="2">
@@ -3653,7 +3653,7 @@
       </s:c>
       <s:c r="C12" s="2" t="inlineStr">
         <s:is>
-          <s:t>香槟瓶</s:t>
+          <s:t>Chocolate Stick</s:t>
         </s:is>
       </s:c>
       <s:c r="D12" s="2">
@@ -3683,7 +3683,7 @@
       </s:c>
       <s:c r="C13" s="2" t="inlineStr">
         <s:is>
-          <s:t>收藏酒瓶</s:t>
+          <s:t>Chocolate Bar</s:t>
         </s:is>
       </s:c>
       <s:c r="D13" s="2">
@@ -3713,7 +3713,7 @@
       </s:c>
       <s:c r="C14" s="2" t="inlineStr">
         <s:is>
-          <s:t>钢钉</s:t>
+          <s:t>Chocolate Drink</s:t>
         </s:is>
       </s:c>
       <s:c r="D14" s="2">
@@ -3743,7 +3743,7 @@
       </s:c>
       <s:c r="C15" s="2" t="inlineStr">
         <s:is>
-          <s:t>药片</s:t>
+          <s:t>Honey Jar</s:t>
         </s:is>
       </s:c>
       <s:c r="D15" s="2">
@@ -3773,7 +3773,7 @@
       </s:c>
       <s:c r="C16" s="2" t="inlineStr">
         <s:is>
-          <s:t>曲奇</s:t>
+          <s:t>Open Honey Jar</s:t>
         </s:is>
       </s:c>
       <s:c r="D16" s="2">
@@ -3804,7 +3804,7 @@
       </s:c>
       <s:c r="C17" s="2" t="inlineStr">
         <s:is>
-          <s:t>苏打饼</s:t>
+          <s:t>Jam Jar</s:t>
         </s:is>
       </s:c>
       <s:c r="D17" s="2">
@@ -3835,7 +3835,7 @@
       </s:c>
       <s:c r="C18" s="2" t="inlineStr">
         <s:is>
-          <s:t>夹心饼</s:t>
+          <s:t>Open Jam Jar</s:t>
         </s:is>
       </s:c>
       <s:c r="D18" s="2">
@@ -3866,7 +3866,7 @@
       </s:c>
       <s:c r="C19" s="2" t="inlineStr">
         <s:is>
-          <s:t>黑巧克力</s:t>
+          <s:t>Bottled Water</s:t>
         </s:is>
       </s:c>
       <s:c r="D19" s="2">
@@ -3897,7 +3897,7 @@
       </s:c>
       <s:c r="C20" s="2" t="inlineStr">
         <s:is>
-          <s:t>牛奶巧克力</s:t>
+          <s:t>Water Bottle with Handle</s:t>
         </s:is>
       </s:c>
       <s:c r="D20" s="2">
@@ -3928,7 +3928,7 @@
       </s:c>
       <s:c r="C21" s="2" t="inlineStr">
         <s:is>
-          <s:t>可可饮料</s:t>
+          <s:t>Large Water Bottle</s:t>
         </s:is>
       </s:c>
       <s:c r="D21" s="2">
@@ -3959,7 +3959,7 @@
       </s:c>
       <s:c r="C22" s="2" t="inlineStr">
         <s:is>
-          <s:t>蜂蜜</s:t>
+          <s:t>Black Canteen</s:t>
         </s:is>
       </s:c>
       <s:c r="D22" s="2">
@@ -3990,7 +3990,7 @@
       </s:c>
       <s:c r="C23" s="2" t="inlineStr">
         <s:is>
-          <s:t>野蜂蜜</s:t>
+          <s:t>Military Canteen</s:t>
         </s:is>
       </s:c>
       <s:c r="D23" s="2">
@@ -4021,7 +4021,7 @@
       </s:c>
       <s:c r="C24" s="2" t="inlineStr">
         <s:is>
-          <s:t>草莓酱</s:t>
+          <s:t>Glass Bottle</s:t>
         </s:is>
       </s:c>
       <s:c r="D24" s="2">
@@ -4052,7 +4052,7 @@
       </s:c>
       <s:c r="C25" s="2" t="inlineStr">
         <s:is>
-          <s:t>蓝莓酱</s:t>
+          <s:t>Round Bottle</s:t>
         </s:is>
       </s:c>
       <s:c r="D25" s="2">
@@ -4083,7 +4083,7 @@
       </s:c>
       <s:c r="C26" s="2" t="inlineStr">
         <s:is>
-          <s:t>肉罐头</s:t>
+          <s:t>Broken Bottle</s:t>
         </s:is>
       </s:c>
       <s:c r="D26" s="2">
@@ -4114,7 +4114,7 @@
       </s:c>
       <s:c r="C27" s="2" t="inlineStr">
         <s:is>
-          <s:t>鱼罐头</s:t>
+          <s:t>Square Bottle</s:t>
         </s:is>
       </s:c>
       <s:c r="D27" s="2">
@@ -4145,7 +4145,7 @@
       </s:c>
       <s:c r="C28" s="2" t="inlineStr">
         <s:is>
-          <s:t>水果罐头</s:t>
+          <s:t>Beer Bottle</s:t>
         </s:is>
       </s:c>
       <s:c r="D28" s="2">
@@ -4176,7 +4176,7 @@
       </s:c>
       <s:c r="C29" s="2" t="inlineStr">
         <s:is>
-          <s:t>午餐肉</s:t>
+          <s:t>Canned Peas</s:t>
         </s:is>
       </s:c>
       <s:c r="D29" s="2">
@@ -4207,7 +4207,7 @@
       </s:c>
       <s:c r="C30" s="2" t="inlineStr">
         <s:is>
-          <s:t>豆子罐头</s:t>
+          <s:t>Open Can of Peas</s:t>
         </s:is>
       </s:c>
       <s:c r="D30" s="2">
@@ -4238,7 +4238,7 @@
       </s:c>
       <s:c r="C31" s="2" t="inlineStr">
         <s:is>
-          <s:t>军粮罐头</s:t>
+          <s:t>Canned Fish</s:t>
         </s:is>
       </s:c>
       <s:c r="D31" s="2">
@@ -4269,7 +4269,7 @@
       </s:c>
       <s:c r="C32" s="2" t="inlineStr">
         <s:is>
-          <s:t>高级罐头</s:t>
+          <s:t>Open Can of Fish</s:t>
         </s:is>
       </s:c>
       <s:c r="D32" s="2">
@@ -4300,7 +4300,7 @@
       </s:c>
       <s:c r="C33" s="2" t="inlineStr">
         <s:is>
-          <s:t>清洁剂</s:t>
+          <s:t>Canned Beans</s:t>
         </s:is>
       </s:c>
       <s:c r="D33" s="2">
@@ -4330,7 +4330,7 @@
       </s:c>
       <s:c r="C34" s="2" t="inlineStr">
         <s:is>
-          <s:t>漂白水</s:t>
+          <s:t>Open Can of Beans</s:t>
         </s:is>
       </s:c>
       <s:c r="D34" s="2">
@@ -4360,7 +4360,7 @@
       </s:c>
       <s:c r="C35" s="2" t="inlineStr">
         <s:is>
-          <s:t>润滑油</s:t>
+          <s:t>Canned Drink</s:t>
         </s:is>
       </s:c>
       <s:c r="D35" s="2">
@@ -4390,7 +4390,7 @@
       </s:c>
       <s:c r="C36" s="2" t="inlineStr">
         <s:is>
-          <s:t>小油壶</s:t>
+          <s:t>Medicine Bottle</s:t>
         </s:is>
       </s:c>
       <s:c r="D36" s="2">
@@ -4421,7 +4421,7 @@
       </s:c>
       <s:c r="C37" s="2" t="inlineStr">
         <s:is>
-          <s:t>运动水壶</s:t>
+          <s:t>Pill Organizer</s:t>
         </s:is>
       </s:c>
       <s:c r="D37" s="2">
@@ -4451,7 +4451,7 @@
       </s:c>
       <s:c r="C38" s="2" t="inlineStr">
         <s:is>
-          <s:t>军用水壶</s:t>
+          <s:t>Syringe</s:t>
         </s:is>
       </s:c>
       <s:c r="D38" s="2">
@@ -4481,7 +4481,7 @@
       </s:c>
       <s:c r="C39" s="2" t="inlineStr">
         <s:is>
-          <s:t>机油壶</s:t>
+          <s:t>Auto-Injector</s:t>
         </s:is>
       </s:c>
       <s:c r="D39" s="2">
@@ -4512,7 +4512,7 @@
       </s:c>
       <s:c r="C40" s="2" t="inlineStr">
         <s:is>
-          <s:t>燃油罐</s:t>
+          <s:t>Bandage Roll</s:t>
         </s:is>
       </s:c>
       <s:c r="D40" s="2">
@@ -4543,7 +4543,7 @@
       </s:c>
       <s:c r="C41" s="2" t="inlineStr">
         <s:is>
-          <s:t>礼帽</s:t>
+          <s:t>IV Bag</s:t>
         </s:is>
       </s:c>
       <s:c r="D41" s="2">
@@ -4573,7 +4573,7 @@
       </s:c>
       <s:c r="C42" s="2" t="inlineStr">
         <s:is>
-          <s:t>棒球帽</s:t>
+          <s:t>First Aid Bag</s:t>
         </s:is>
       </s:c>
       <s:c r="D42" s="2">
@@ -4603,7 +4603,7 @@
       </s:c>
       <s:c r="C43" s="2" t="inlineStr">
         <s:is>
-          <s:t>墨镜</s:t>
+          <s:t>First Aid Kit</s:t>
         </s:is>
       </s:c>
       <s:c r="D43" s="2">
@@ -4633,7 +4633,7 @@
       </s:c>
       <s:c r="C44" s="2" t="inlineStr">
         <s:is>
-          <s:t>太阳镜</s:t>
+          <s:t>Medical Case</s:t>
         </s:is>
       </s:c>
       <s:c r="D44" s="2">
@@ -4663,7 +4663,7 @@
       </s:c>
       <s:c r="C45" s="2" t="inlineStr">
         <s:is>
-          <s:t>护目镜</s:t>
+          <s:t>Cleaning Spray</s:t>
         </s:is>
       </s:c>
       <s:c r="D45" s="2">
@@ -4693,7 +4693,7 @@
       </s:c>
       <s:c r="C46" s="2" t="inlineStr">
         <s:is>
-          <s:t>战术风镜</s:t>
+          <s:t>Bleach</s:t>
         </s:is>
       </s:c>
       <s:c r="D46" s="2">
@@ -4723,7 +4723,7 @@
       </s:c>
       <s:c r="C47" s="2" t="inlineStr">
         <s:is>
-          <s:t>口罩</s:t>
+          <s:t>Lubricant Spray</s:t>
         </s:is>
       </s:c>
       <s:c r="D47" s="2">
@@ -4753,7 +4753,7 @@
       </s:c>
       <s:c r="C48" s="2" t="inlineStr">
         <s:is>
-          <s:t>防毒面具</s:t>
+          <s:t>Metal Pipe</s:t>
         </s:is>
       </s:c>
       <s:c r="D48" s="2">
@@ -4783,7 +4783,7 @@
       </s:c>
       <s:c r="C49" s="2" t="inlineStr">
         <s:is>
-          <s:t>战术面具</s:t>
+          <s:t>Flip-Top Lighter</s:t>
         </s:is>
       </s:c>
       <s:c r="D49" s="2">
@@ -4813,7 +4813,7 @@
       </s:c>
       <s:c r="C50" s="2" t="inlineStr">
         <s:is>
-          <s:t>皮靴</s:t>
+          <s:t>Red Fuel Can</s:t>
         </s:is>
       </s:c>
       <s:c r="D50" s="2">
@@ -4843,7 +4843,7 @@
       </s:c>
       <s:c r="C51" s="2" t="inlineStr">
         <s:is>
-          <s:t>雨靴</s:t>
+          <s:t>Green Fuel Can</s:t>
         </s:is>
       </s:c>
       <s:c r="D51" s="2">
@@ -4873,7 +4873,7 @@
       </s:c>
       <s:c r="C52" s="2" t="inlineStr">
         <s:is>
-          <s:t>登山靴</s:t>
+          <s:t>Jerry Can</s:t>
         </s:is>
       </s:c>
       <s:c r="D52" s="2">
@@ -4903,7 +4903,7 @@
       </s:c>
       <s:c r="C53" s="2" t="inlineStr">
         <s:is>
-          <s:t>军靴</s:t>
+          <s:t>Smartphone</s:t>
         </s:is>
       </s:c>
       <s:c r="D53" s="2">
@@ -4933,7 +4933,7 @@
       </s:c>
       <s:c r="C54" s="2" t="inlineStr">
         <s:is>
-          <s:t>防弹背心</s:t>
+          <s:t>Stopwatch</s:t>
         </s:is>
       </s:c>
       <s:c r="D54" s="2">
@@ -4963,7 +4963,7 @@
       </s:c>
       <s:c r="C55" s="2" t="inlineStr">
         <s:is>
-          <s:t>重型护甲</s:t>
+          <s:t>Pet ID Tag</s:t>
         </s:is>
       </s:c>
       <s:c r="D55" s="2">
@@ -4993,7 +4993,7 @@
       </s:c>
       <s:c r="C56" s="2" t="inlineStr">
         <s:is>
-          <s:t>工地头盔</s:t>
+          <s:t>Compass</s:t>
         </s:is>
       </s:c>
       <s:c r="D56" s="2">
@@ -5023,7 +5023,7 @@
       </s:c>
       <s:c r="C57" s="2" t="inlineStr">
         <s:is>
-          <s:t>骑行头盔</s:t>
+          <s:t>Folding Compass</s:t>
         </s:is>
       </s:c>
       <s:c r="D57" s="2">
@@ -5053,7 +5053,7 @@
       </s:c>
       <s:c r="C58" s="2" t="inlineStr">
         <s:is>
-          <s:t>防暴头盔</s:t>
+          <s:t>Fedora</s:t>
         </s:is>
       </s:c>
       <s:c r="D58" s="2">
@@ -5083,7 +5083,7 @@
       </s:c>
       <s:c r="C59" s="2" t="inlineStr">
         <s:is>
-          <s:t>战术头盔</s:t>
+          <s:t>Baseball Cap</s:t>
         </s:is>
       </s:c>
       <s:c r="D59" s="2">
@@ -5113,7 +5113,7 @@
       </s:c>
       <s:c r="C60" s="2" t="inlineStr">
         <s:is>
-          <s:t>小背包</s:t>
+          <s:t>Gold-Framed Sunglasses</s:t>
         </s:is>
       </s:c>
       <s:c r="D60" s="2">
@@ -5143,7 +5143,7 @@
       </s:c>
       <s:c r="C61" s="2" t="inlineStr">
         <s:is>
-          <s:t>登山包</s:t>
+          <s:t>Sunglasses</s:t>
         </s:is>
       </s:c>
       <s:c r="D61" s="2">
@@ -5173,7 +5173,7 @@
       </s:c>
       <s:c r="C62" s="2" t="inlineStr">
         <s:is>
-          <s:t>军用背包</s:t>
+          <s:t>Safety Goggles</s:t>
         </s:is>
       </s:c>
       <s:c r="D62" s="2">
@@ -5203,7 +5203,7 @@
       </s:c>
       <s:c r="C63" s="2" t="inlineStr">
         <s:is>
-          <s:t>铁锅</s:t>
+          <s:t>Tactical Goggles</s:t>
         </s:is>
       </s:c>
       <s:c r="D63" s="2">
@@ -5233,7 +5233,7 @@
       </s:c>
       <s:c r="C64" s="2" t="inlineStr">
         <s:is>
-          <s:t>木锤</s:t>
+          <s:t>Dust Mask</s:t>
         </s:is>
       </s:c>
       <s:c r="D64" s="2">
@@ -5263,7 +5263,7 @@
       </s:c>
       <s:c r="C65" s="2" t="inlineStr">
         <s:is>
-          <s:t>铁锤</s:t>
+          <s:t>Half-Face Respirator</s:t>
         </s:is>
       </s:c>
       <s:c r="D65" s="2">
@@ -5293,7 +5293,7 @@
       </s:c>
       <s:c r="C66" s="2" t="inlineStr">
         <s:is>
-          <s:t>大锤</s:t>
+          <s:t>Gas Mask</s:t>
         </s:is>
       </s:c>
       <s:c r="D66" s="2">
@@ -5323,7 +5323,7 @@
       </s:c>
       <s:c r="C67" s="2" t="inlineStr">
         <s:is>
-          <s:t>扳手</s:t>
+          <s:t>Brown Boots</s:t>
         </s:is>
       </s:c>
       <s:c r="D67" s="2">
@@ -5353,7 +5353,7 @@
       </s:c>
       <s:c r="C68" s="2" t="inlineStr">
         <s:is>
-          <s:t>活动扳手</s:t>
+          <s:t>Black Boots</s:t>
         </s:is>
       </s:c>
       <s:c r="D68" s="2">
@@ -5383,7 +5383,7 @@
       </s:c>
       <s:c r="C69" s="2" t="inlineStr">
         <s:is>
-          <s:t>管钳</s:t>
+          <s:t>Rubber Boots</s:t>
         </s:is>
       </s:c>
       <s:c r="D69" s="2">
@@ -5413,7 +5413,7 @@
       </s:c>
       <s:c r="C70" s="2" t="inlineStr">
         <s:is>
-          <s:t>工兵铲</s:t>
+          <s:t>Leather Shoes</s:t>
         </s:is>
       </s:c>
       <s:c r="D70" s="2">
@@ -5443,7 +5443,7 @@
       </s:c>
       <s:c r="C71" s="2" t="inlineStr">
         <s:is>
-          <s:t>铁锹</s:t>
+          <s:t>Bulletproof Vest</s:t>
         </s:is>
       </s:c>
       <s:c r="D71" s="2">
@@ -5473,7 +5473,7 @@
       </s:c>
       <s:c r="C72" s="2" t="inlineStr">
         <s:is>
-          <s:t>十字镐</s:t>
+          <s:t>Heavy Armor Vest</s:t>
         </s:is>
       </s:c>
       <s:c r="D72" s="2">
@@ -5503,7 +5503,7 @@
       </s:c>
       <s:c r="C73" s="2" t="inlineStr">
         <s:is>
-          <s:t>胶囊</s:t>
+          <s:t>Helmet with Goggles</s:t>
         </s:is>
       </s:c>
       <s:c r="D73" s="2">
@@ -5533,7 +5533,7 @@
       </s:c>
       <s:c r="C74" s="2" t="inlineStr">
         <s:is>
-          <s:t>干电池</s:t>
+          <s:t>Combat Helmet</s:t>
         </s:is>
       </s:c>
       <s:c r="D74" s="2">
@@ -5563,7 +5563,7 @@
       </s:c>
       <s:c r="C75" s="2" t="inlineStr">
         <s:is>
-          <s:t>强力电池</s:t>
+          <s:t>Riot Helmet</s:t>
         </s:is>
       </s:c>
       <s:c r="D75" s="2">
@@ -5593,7 +5593,7 @@
       </s:c>
       <s:c r="C76" s="2" t="inlineStr">
         <s:is>
-          <s:t>药瓶</s:t>
+          <s:t>Tactical Helmet</s:t>
         </s:is>
       </s:c>
       <s:c r="D76" s="2">
@@ -5623,7 +5623,7 @@
       </s:c>
       <s:c r="C77" s="2" t="inlineStr">
         <s:is>
-          <s:t>急救药瓶</s:t>
+          <s:t>Multi-Pocket Backpack</s:t>
         </s:is>
       </s:c>
       <s:c r="D77" s="2">
@@ -5653,7 +5653,7 @@
       </s:c>
       <s:c r="C78" s="2" t="inlineStr">
         <s:is>
-          <s:t>注射器</s:t>
+          <s:t>Tactical Backpack</s:t>
         </s:is>
       </s:c>
       <s:c r="D78" s="2">
@@ -5683,7 +5683,7 @@
       </s:c>
       <s:c r="C79" s="2" t="inlineStr">
         <s:is>
-          <s:t>强化针</s:t>
+          <s:t>Large Tactical Backpack</s:t>
         </s:is>
       </s:c>
       <s:c r="D79" s="2">
@@ -5713,7 +5713,7 @@
       </s:c>
       <s:c r="C80" s="2" t="inlineStr">
         <s:is>
-          <s:t>医用绷带</s:t>
+          <s:t>Toolbox</s:t>
         </s:is>
       </s:c>
       <s:c r="D80" s="2">
@@ -5743,7 +5743,7 @@
       </s:c>
       <s:c r="C81" s="2" t="inlineStr">
         <s:is>
-          <s:t>绿色徽章</s:t>
+          <s:t>Supply Case</s:t>
         </s:is>
       </s:c>
       <s:c r="D81" s="2">
@@ -5773,7 +5773,7 @@
       </s:c>
       <s:c r="C82" s="2" t="inlineStr">
         <s:is>
-          <s:t>急救包</s:t>
+          <s:t>Equipment Case</s:t>
         </s:is>
       </s:c>
       <s:c r="D82" s="2">
@@ -5803,7 +5803,7 @@
       </s:c>
       <s:c r="C83" s="2" t="inlineStr">
         <s:is>
-          <s:t>医疗箱</s:t>
+          <s:t>Cooking Pot</s:t>
         </s:is>
       </s:c>
       <s:c r="D83" s="2">
@@ -5833,7 +5833,7 @@
       </s:c>
       <s:c r="C84" s="2" t="inlineStr">
         <s:is>
-          <s:t>高级医疗箱</s:t>
+          <s:t>Red Barrel</s:t>
         </s:is>
       </s:c>
       <s:c r="D84" s="2">
@@ -5863,7 +5863,7 @@
       </s:c>
       <s:c r="C85" s="2" t="inlineStr">
         <s:is>
-          <s:t>钢管</s:t>
+          <s:t>Blue Barrel</s:t>
         </s:is>
       </s:c>
       <s:c r="D85" s="2">
@@ -5893,7 +5893,7 @@
       </s:c>
       <s:c r="C86" s="2" t="inlineStr">
         <s:is>
-          <s:t>手机</s:t>
+          <s:t>Sealed Drum</s:t>
         </s:is>
       </s:c>
       <s:c r="D86" s="2">
@@ -5923,7 +5923,7 @@
       </s:c>
       <s:c r="C87" s="2" t="inlineStr">
         <s:is>
-          <s:t>手表</s:t>
+          <s:t>Blue Steel Drum</s:t>
         </s:is>
       </s:c>
       <s:c r="D87" s="2">
@@ -5953,7 +5953,7 @@
       </s:c>
       <s:c r="C88" s="2" t="inlineStr">
         <s:is>
-          <s:t>身份牌</s:t>
+          <s:t>Hazardous Materials Drum</s:t>
         </s:is>
       </s:c>
       <s:c r="D88" s="2">
@@ -5983,7 +5983,7 @@
       </s:c>
       <s:c r="C89" s="2" t="inlineStr">
         <s:is>
-          <s:t>指南针</s:t>
+          <s:t>Propane Tank</s:t>
         </s:is>
       </s:c>
       <s:c r="D89" s="2">
@@ -6013,7 +6013,7 @@
       </s:c>
       <s:c r="C90" s="2" t="inlineStr">
         <s:is>
-          <s:t>军用罗盘</s:t>
+          <s:t>Rope</s:t>
         </s:is>
       </s:c>
       <s:c r="D90" s="2">
@@ -6043,7 +6043,7 @@
       </s:c>
       <s:c r="C91" s="2" t="inlineStr">
         <s:is>
-          <s:t>木箱</s:t>
+          <s:t>Wire Coil</s:t>
         </s:is>
       </s:c>
       <s:c r="D91" s="2">
@@ -6073,7 +6073,7 @@
       </s:c>
       <s:c r="C92" s="2" t="inlineStr">
         <s:is>
-          <s:t>工具箱</s:t>
+          <s:t>Walkie-Talkie</s:t>
         </s:is>
       </s:c>
       <s:c r="D92" s="2">
@@ -6103,7 +6103,7 @@
       </s:c>
       <s:c r="C93" s="2" t="inlineStr">
         <s:is>
-          <s:t>补给箱</s:t>
+          <s:t>Field Radio</s:t>
         </s:is>
       </s:c>
       <s:c r="D93" s="2">
@@ -6133,7 +6133,7 @@
       </s:c>
       <s:c r="C94" s="2" t="inlineStr">
         <s:is>
-          <s:t>油桶</s:t>
+          <s:t>Flashlight</s:t>
         </s:is>
       </s:c>
       <s:c r="D94" s="2">
@@ -6163,7 +6163,7 @@
       </s:c>
       <s:c r="C95" s="2" t="inlineStr">
         <s:is>
-          <s:t>储物桶</s:t>
+          <s:t>Headlamp</s:t>
         </s:is>
       </s:c>
       <s:c r="D95" s="2">
@@ -6193,7 +6193,7 @@
       </s:c>
       <s:c r="C96" s="2" t="inlineStr">
         <s:is>
-          <s:t>密封桶</s:t>
+          <s:t>Lantern</s:t>
         </s:is>
       </s:c>
       <s:c r="D96" s="2">
@@ -6223,7 +6223,7 @@
       </s:c>
       <s:c r="C97" s="2" t="inlineStr">
         <s:is>
-          <s:t>大铁桶</s:t>
+          <s:t>Telescope</s:t>
         </s:is>
       </s:c>
       <s:c r="D97" s="2">
@@ -6253,7 +6253,7 @@
       </s:c>
       <s:c r="C98" s="2" t="inlineStr">
         <s:is>
-          <s:t>煤气罐</s:t>
+          <s:t>Binoculars</s:t>
         </s:is>
       </s:c>
       <s:c r="D98" s="2">
@@ -6283,7 +6283,7 @@
       </s:c>
       <s:c r="C99" s="2" t="inlineStr">
         <s:is>
-          <s:t>粗绳</s:t>
+          <s:t>Claw Hammer</s:t>
         </s:is>
       </s:c>
       <s:c r="D99" s="2">
@@ -6313,7 +6313,7 @@
       </s:c>
       <s:c r="C100" s="2" t="inlineStr">
         <s:is>
-          <s:t>电线</s:t>
+          <s:t>Hammer</s:t>
         </s:is>
       </s:c>
       <s:c r="D100" s="2">
@@ -6343,7 +6343,7 @@
       </s:c>
       <s:c r="C101" s="2" t="inlineStr">
         <s:is>
-          <s:t>对讲机</s:t>
+          <s:t>Sledgehammer</s:t>
         </s:is>
       </s:c>
       <s:c r="D101" s="2">
@@ -6373,7 +6373,7 @@
       </s:c>
       <s:c r="C102" s="2" t="inlineStr">
         <s:is>
-          <s:t>军用电台</s:t>
+          <s:t>Adjustable Wrench</s:t>
         </s:is>
       </s:c>
       <s:c r="D102" s="2">
@@ -6403,7 +6403,7 @@
       </s:c>
       <s:c r="C103" s="2" t="inlineStr">
         <s:is>
-          <s:t>手电筒</s:t>
+          <s:t>Pipe Wrench</s:t>
         </s:is>
       </s:c>
       <s:c r="D103" s="2">
@@ -6433,7 +6433,7 @@
       </s:c>
       <s:c r="C104" s="2" t="inlineStr">
         <s:is>
-          <s:t>头灯</s:t>
+          <s:t>Crowbar</s:t>
         </s:is>
       </s:c>
       <s:c r="D104" s="2">
@@ -6463,7 +6463,7 @@
       </s:c>
       <s:c r="C105" s="2" t="inlineStr">
         <s:is>
-          <s:t>提灯</s:t>
+          <s:t>Entrenching Shovel</s:t>
         </s:is>
       </s:c>
       <s:c r="D105" s="2">
@@ -6493,7 +6493,7 @@
       </s:c>
       <s:c r="C106" s="2" t="inlineStr">
         <s:is>
-          <s:t>望远镜</s:t>
+          <s:t>Shovel</s:t>
         </s:is>
       </s:c>
       <s:c r="D106" s="2">
@@ -6523,7 +6523,7 @@
       </s:c>
       <s:c r="C107" s="2" t="inlineStr">
         <s:is>
-          <s:t>高倍望远镜</s:t>
+          <s:t>Pickaxe</s:t>
         </s:is>
       </s:c>
       <s:c r="D107" s="2">
@@ -6553,7 +6553,7 @@
       </s:c>
       <s:c r="C108" s="2" t="inlineStr">
         <s:is>
-          <s:t>高尔夫球杆</s:t>
+          <s:t>Croquet Mallet</s:t>
         </s:is>
       </s:c>
       <s:c r="D108" s="2" t="n">
@@ -6583,7 +6583,7 @@
       </s:c>
       <s:c r="C109" s="2" t="inlineStr">
         <s:is>
-          <s:t>冰球杆</s:t>
+          <s:t>Hockey Stick</s:t>
         </s:is>
       </s:c>
       <s:c r="D109" s="2" t="n">
@@ -6613,7 +6613,7 @@
       </s:c>
       <s:c r="C110" s="2" t="inlineStr">
         <s:is>
-          <s:t>木棒</s:t>
+          <s:t>Wooden Baseball Bat</s:t>
         </s:is>
       </s:c>
       <s:c r="D110" s="2" t="n">
@@ -6643,7 +6643,7 @@
       </s:c>
       <s:c r="C111" s="2" t="inlineStr">
         <s:is>
-          <s:t>球棒</s:t>
+          <s:t>Metal Baseball Bat</s:t>
         </s:is>
       </s:c>
       <s:c r="D111" s="2" t="n">
@@ -6673,7 +6673,7 @@
       </s:c>
       <s:c r="C112" s="2" t="inlineStr">
         <s:is>
-          <s:t>铁棒</s:t>
+          <s:t>Spiked Metal Bat</s:t>
         </s:is>
       </s:c>
       <s:c r="D112" s="2" t="n">
@@ -6703,7 +6703,7 @@
       </s:c>
       <s:c r="C113" s="2" t="inlineStr">
         <s:is>
-          <s:t>战术棍</s:t>
+          <s:t>Nailed Wooden Bat</s:t>
         </s:is>
       </s:c>
       <s:c r="D113" s="2" t="n">
@@ -6733,7 +6733,7 @@
       </s:c>
       <s:c r="C114" s="2" t="inlineStr">
         <s:is>
-          <s:t>电锯</s:t>
+          <s:t>Chainsaw</s:t>
         </s:is>
       </s:c>
       <s:c r="D114" s="2" t="n">
@@ -6763,7 +6763,7 @@
       </s:c>
       <s:c r="C115" s="2" t="inlineStr">
         <s:is>
-          <s:t>木斧</s:t>
+          <s:t>Hatchet</s:t>
         </s:is>
       </s:c>
       <s:c r="D115" s="2" t="n">
@@ -6793,7 +6793,7 @@
       </s:c>
       <s:c r="C116" s="2" t="inlineStr">
         <s:is>
-          <s:t>消防斧</s:t>
+          <s:t>Chopping Axe</s:t>
         </s:is>
       </s:c>
       <s:c r="D116" s="2" t="n">
@@ -6823,7 +6823,7 @@
       </s:c>
       <s:c r="C117" s="2" t="inlineStr">
         <s:is>
-          <s:t>战斧</s:t>
+          <s:t>Double-Bladed Battle Axe</s:t>
         </s:is>
       </s:c>
       <s:c r="D117" s="2" t="n">
@@ -6853,7 +6853,7 @@
       </s:c>
       <s:c r="C118" s="2" t="inlineStr">
         <s:is>
-          <s:t>小刀</s:t>
+          <s:t>Knife</s:t>
         </s:is>
       </s:c>
       <s:c r="D118" s="2" t="n">
@@ -6883,7 +6883,7 @@
       </s:c>
       <s:c r="C119" s="2" t="inlineStr">
         <s:is>
-          <s:t>猎刀</s:t>
+          <s:t>Hunting Knife</s:t>
         </s:is>
       </s:c>
       <s:c r="D119" s="2" t="n">
@@ -6913,7 +6913,7 @@
       </s:c>
       <s:c r="C120" s="2" t="inlineStr">
         <s:is>
-          <s:t>军刀</s:t>
+          <s:t>Knuckle Knife</s:t>
         </s:is>
       </s:c>
       <s:c r="D120" s="2" t="n">
@@ -6943,7 +6943,7 @@
       </s:c>
       <s:c r="C121" s="2" t="inlineStr">
         <s:is>
-          <s:t>开山刀</s:t>
+          <s:t>Karambit</s:t>
         </s:is>
       </s:c>
       <s:c r="D121" s="2" t="n">
@@ -6973,7 +6973,7 @@
       </s:c>
       <s:c r="C122" s="2" t="inlineStr">
         <s:is>
-          <s:t>匕首</s:t>
+          <s:t>Cleaver</s:t>
         </s:is>
       </s:c>
       <s:c r="D122" s="2" t="n">
@@ -7003,7 +7003,7 @@
       </s:c>
       <s:c r="C123" s="2" t="inlineStr">
         <s:is>
-          <s:t>战术刀</s:t>
+          <s:t>Machete</s:t>
         </s:is>
       </s:c>
       <s:c r="D123" s="2" t="n">
@@ -7033,7 +7033,7 @@
       </s:c>
       <s:c r="C124" s="2" t="inlineStr">
         <s:is>
-          <s:t>狼牙棒</s:t>
+          <s:t>Spiked Mace</s:t>
         </s:is>
       </s:c>
       <s:c r="D124" s="2" t="n">
@@ -7063,7 +7063,7 @@
       </s:c>
       <s:c r="C125" s="6" t="inlineStr">
         <s:is>
-          <s:t>炸药罐</s:t>
+          <s:t>Dynamite Stick</s:t>
         </s:is>
       </s:c>
       <s:c r="D125" s="2" t="n">
@@ -7092,7 +7092,7 @@
       </s:c>
       <s:c r="C126" s="6" t="inlineStr">
         <s:is>
-          <s:t>捆装炸药</s:t>
+          <s:t>Dynamite Bundle</s:t>
         </s:is>
       </s:c>
       <s:c r="D126" s="2" t="n">
@@ -7121,7 +7121,7 @@
       </s:c>
       <s:c r="C127" s="6" t="inlineStr">
         <s:is>
-          <s:t>遥控炸弹</s:t>
+          <s:t>Dynamite with Detonator</s:t>
         </s:is>
       </s:c>
       <s:c r="D127" s="2" t="n">
@@ -7150,7 +7150,7 @@
       </s:c>
       <s:c r="C128" s="6" t="inlineStr">
         <s:is>
-          <s:t>圆形手雷</s:t>
+          <s:t>Round Grenade</s:t>
         </s:is>
       </s:c>
       <s:c r="D128" s="2" t="n">
@@ -7179,7 +7179,7 @@
       </s:c>
       <s:c r="C129" s="6" t="inlineStr">
         <s:is>
-          <s:t>高爆手雷</s:t>
+          <s:t>Canister Grenade</s:t>
         </s:is>
       </s:c>
       <s:c r="D129" s="2" t="n">
@@ -7208,7 +7208,7 @@
       </s:c>
       <s:c r="C130" s="6" t="inlineStr">
         <s:is>
-          <s:t>等离子手雷</s:t>
+          <s:t>Energy Grenade</s:t>
         </s:is>
       </s:c>
       <s:c r="D130" s="2" t="n">
@@ -7237,7 +7237,7 @@
       </s:c>
       <s:c r="C131" s="6" t="inlineStr">
         <s:is>
-          <s:t>感应地雷</s:t>
+          <s:t>Land Mine</s:t>
         </s:is>
       </s:c>
       <s:c r="D131" s="2" t="n">
@@ -7266,7 +7266,7 @@
       </s:c>
       <s:c r="C132" s="6" t="inlineStr">
         <s:is>
-          <s:t>捕兽夹</s:t>
+          <s:t>Bear Trap</s:t>
         </s:is>
       </s:c>
       <s:c r="D132" s="2" t="n">
@@ -7295,7 +7295,7 @@
       </s:c>
       <s:c r="C133" s="6" t="inlineStr">
         <s:is>
-          <s:t>手枪子弹</s:t>
+          <s:t>Pistol Round</s:t>
         </s:is>
       </s:c>
       <s:c r="D133" s="2" t="n">
@@ -7324,7 +7324,7 @@
       </s:c>
       <s:c r="C134" s="6" t="inlineStr">
         <s:is>
-          <s:t>手枪弹药</s:t>
+          <s:t>Pistol Ammo</s:t>
         </s:is>
       </s:c>
       <s:c r="D134" s="2" t="n">
@@ -7353,7 +7353,7 @@
       </s:c>
       <s:c r="C135" s="6" t="inlineStr">
         <s:is>
-          <s:t>整箱弹药</s:t>
+          <s:t>Ammo Crate</s:t>
         </s:is>
       </s:c>
       <s:c r="D135" s="2" t="n">
@@ -7382,7 +7382,7 @@
       </s:c>
       <s:c r="C136" s="6" t="inlineStr">
         <s:is>
-          <s:t>盒装弹药</s:t>
+          <s:t>Boxed Ammo</s:t>
         </s:is>
       </s:c>
       <s:c r="D136" s="2" t="n">
@@ -7411,7 +7411,7 @@
       </s:c>
       <s:c r="C137" s="6" t="inlineStr">
         <s:is>
-          <s:t>直式弹匣</s:t>
+          <s:t>Straight Magazine</s:t>
         </s:is>
       </s:c>
       <s:c r="D137" s="2" t="n">
@@ -7440,7 +7440,7 @@
       </s:c>
       <s:c r="C138" s="6" t="inlineStr">
         <s:is>
-          <s:t>弯式弹匣</s:t>
+          <s:t>Curved Magazine</s:t>
         </s:is>
       </s:c>
       <s:c r="D138" s="2" t="n">
@@ -7469,7 +7469,7 @@
       </s:c>
       <s:c r="C139" s="6" t="inlineStr">
         <s:is>
-          <s:t>霰弹盒</s:t>
+          <s:t>Pellet Box</s:t>
         </s:is>
       </s:c>
       <s:c r="D139" s="2" t="n">
@@ -7498,7 +7498,7 @@
       </s:c>
       <s:c r="C140" s="6" t="inlineStr">
         <s:is>
-          <s:t>军用弹药箱</s:t>
+          <s:t>Military Ammo Can</s:t>
         </s:is>
       </s:c>
       <s:c r="D140" s="2" t="n">
@@ -7527,7 +7527,7 @@
       </s:c>
       <s:c r="C141" s="6" t="inlineStr">
         <s:is>
-          <s:t>左轮手枪</s:t>
+          <s:t>Revolver</s:t>
         </s:is>
       </s:c>
       <s:c r="D141" s="2" t="n">
@@ -7556,7 +7556,7 @@
       </s:c>
       <s:c r="C142" s="6" t="inlineStr">
         <s:is>
-          <s:t>单发手枪</s:t>
+          <s:t>Single-Shot Pistol</s:t>
         </s:is>
       </s:c>
       <s:c r="D142" s="2" t="n">
@@ -7585,7 +7585,7 @@
       </s:c>
       <s:c r="C143" s="6" t="inlineStr">
         <s:is>
-          <s:t>短管突击步枪</s:t>
+          <s:t>Short-Barreled Assault Rifle</s:t>
         </s:is>
       </s:c>
       <s:c r="D143" s="2" t="n">
@@ -7614,7 +7614,7 @@
       </s:c>
       <s:c r="C144" s="6" t="inlineStr">
         <s:is>
-          <s:t>战术突击步枪</s:t>
+          <s:t>Folding-Stock Assault Rifle</s:t>
         </s:is>
       </s:c>
       <s:c r="D144" s="2" t="n">
@@ -7643,7 +7643,7 @@
       </s:c>
       <s:c r="C145" s="6" t="inlineStr">
         <s:is>
-          <s:t>木托突击步枪</s:t>
+          <s:t>Wooden-Stock Assault Rifle</s:t>
         </s:is>
       </s:c>
       <s:c r="D145" s="2" t="n">
@@ -7672,7 +7672,7 @@
       </s:c>
       <s:c r="C146" s="6" t="inlineStr">
         <s:is>
-          <s:t>战斗霰弹枪</s:t>
+          <s:t>Grenade Launcher</s:t>
         </s:is>
       </s:c>
       <s:c r="D146" s="2" t="n">
@@ -7701,7 +7701,7 @@
       </s:c>
       <s:c r="C147" s="6" t="inlineStr">
         <s:is>
-          <s:t>狙击步枪</s:t>
+          <s:t>Sniper Rifle</s:t>
         </s:is>
       </s:c>
       <s:c r="D147" s="2" t="n">
@@ -7730,7 +7730,7 @@
       </s:c>
       <s:c r="C148" s="6" t="inlineStr">
         <s:is>
-          <s:t>冲锋枪</s:t>
+          <s:t>Submachine Gun</s:t>
         </s:is>
       </s:c>
       <s:c r="D148" s="2" t="n">
@@ -7759,7 +7759,7 @@
       </s:c>
       <s:c r="C149" s="6" t="inlineStr">
         <s:is>
-          <s:t>消音冲锋枪</s:t>
+          <s:t>Suppressed Submachine Gun</s:t>
         </s:is>
       </s:c>
       <s:c r="D149" s="2" t="n">
@@ -7788,7 +7788,7 @@
       </s:c>
       <s:c r="C150" s="6" t="inlineStr">
         <s:is>
-          <s:t>微型冲锋枪</s:t>
+          <s:t>Compact Submachine Gun</s:t>
         </s:is>
       </s:c>
       <s:c r="D150" s="2" t="n">
@@ -7817,7 +7817,7 @@
       </s:c>
       <s:c r="C151" s="6" t="inlineStr">
         <s:is>
-          <s:t>木托冲锋枪</s:t>
+          <s:t>Wooden-Stock Submachine Gun</s:t>
         </s:is>
       </s:c>
       <s:c r="D151" s="2" t="n">

</xml_diff>